<commit_message>
data: actualizar outputs con corrida 2026-03-12
399K leads, codcar ingreso reclasificados a Grado_Pregrado (+770 insc),
nuevos leads dic/ene incorporados. Excluidos 2 xlsx >30MB.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing_report/outputs/Auditoria_Indicadores/Auditoria_Indicadores.xlsx
+++ b/marketing_report/outputs/Auditoria_Indicadores/Auditoria_Indicadores.xlsx
@@ -504,16 +504,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>369148</v>
+        <v>398556</v>
       </c>
       <c r="C2" t="n">
-        <v>965</v>
+        <v>44</v>
       </c>
       <c r="D2" t="n">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="E2" t="n">
-        <v>370270</v>
+        <v>398778</v>
       </c>
     </row>
     <row r="3">
@@ -523,16 +523,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11468</v>
+        <v>13170</v>
       </c>
       <c r="C3" t="n">
-        <v>941</v>
+        <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="E3" t="n">
-        <v>12532</v>
+        <v>13343</v>
       </c>
     </row>
     <row r="4">
@@ -542,16 +542,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="C4" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E4" t="n">
-        <v>246</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>357492</v>
+        <v>385231</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -570,7 +570,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>357492</v>
+        <v>385231</v>
       </c>
     </row>
     <row r="6">
@@ -580,16 +580,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>369148</v>
+        <v>398556</v>
       </c>
       <c r="C6" t="n">
-        <v>965</v>
+        <v>44</v>
       </c>
       <c r="D6" t="n">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="E6" t="n">
-        <v>370270</v>
+        <v>398778</v>
       </c>
     </row>
     <row r="7">
@@ -599,16 +599,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>286660</v>
+        <v>305249</v>
       </c>
       <c r="C7" t="n">
-        <v>616</v>
+        <v>25</v>
       </c>
       <c r="D7" t="n">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="E7" t="n">
-        <v>287403</v>
+        <v>305419</v>
       </c>
     </row>
     <row r="8">
@@ -618,16 +618,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7020</v>
+        <v>7980</v>
       </c>
       <c r="C8" t="n">
-        <v>592</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E8" t="n">
-        <v>7705</v>
+        <v>8101</v>
       </c>
     </row>
     <row r="9">
@@ -637,16 +637,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="C9" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E9" t="n">
-        <v>246</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>279452</v>
+        <v>297114</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>279452</v>
+        <v>297114</v>
       </c>
     </row>
     <row r="11">
@@ -675,16 +675,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>286660</v>
+        <v>305249</v>
       </c>
       <c r="C11" t="n">
-        <v>616</v>
+        <v>25</v>
       </c>
       <c r="D11" t="n">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="E11" t="n">
-        <v>287403</v>
+        <v>305419</v>
       </c>
     </row>
     <row r="12">
@@ -738,16 +738,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>152231</v>
+        <v>170085</v>
       </c>
       <c r="C14" t="n">
-        <v>600</v>
+        <v>21</v>
       </c>
       <c r="D14" t="n">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="E14" t="n">
-        <v>152936</v>
+        <v>170229</v>
       </c>
     </row>
     <row r="15">
@@ -757,16 +757,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5892</v>
+        <v>6911</v>
       </c>
       <c r="C15" t="n">
-        <v>581</v>
+        <v>18</v>
       </c>
       <c r="D15" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="E15" t="n">
-        <v>6550</v>
+        <v>7013</v>
       </c>
     </row>
     <row r="16">
@@ -776,16 +776,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.8704</v>
+        <v>4.0633</v>
       </c>
       <c r="C16" t="n">
-        <v>96.83329999999999</v>
+        <v>85.71429999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>73.33329999999999</v>
+        <v>68.2927</v>
       </c>
       <c r="E16" t="n">
-        <v>174.037</v>
+        <v>158.0703</v>
       </c>
     </row>
     <row r="17">
@@ -795,10 +795,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8755</v>
+        <v>9525</v>
       </c>
       <c r="C17" t="n">
-        <v>864</v>
+        <v>94</v>
       </c>
       <c r="D17" t="n">
         <v>325</v>
@@ -814,16 +814,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6926</v>
+        <v>7993</v>
       </c>
       <c r="C18" t="n">
-        <v>572</v>
+        <v>19</v>
       </c>
       <c r="D18" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E18" t="n">
-        <v>7550</v>
+        <v>8070</v>
       </c>
     </row>
     <row r="19">
@@ -833,16 +833,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1641</v>
+        <v>1377</v>
       </c>
       <c r="C19" t="n">
-        <v>268</v>
+        <v>71</v>
       </c>
       <c r="D19" t="n">
-        <v>239</v>
+        <v>222</v>
       </c>
       <c r="E19" t="n">
-        <v>2148</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="20">
@@ -852,16 +852,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>18436</v>
+        <v>20504</v>
       </c>
       <c r="C20" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E20" t="n">
-        <v>18492</v>
+        <v>20526</v>
       </c>
     </row>
     <row r="21">
@@ -871,16 +871,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>970</v>
+        <v>1117</v>
       </c>
       <c r="C21" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>1014</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="22">
@@ -890,16 +890,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>111503</v>
+        <v>123201</v>
       </c>
       <c r="C22" t="n">
-        <v>139</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="E22" t="n">
-        <v>111703</v>
+        <v>123286</v>
       </c>
     </row>
     <row r="23">
@@ -909,16 +909,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>821</v>
+        <v>880</v>
       </c>
       <c r="C23" t="n">
-        <v>132</v>
+        <v>8</v>
       </c>
       <c r="D23" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E23" t="n">
-        <v>997</v>
+        <v>936</v>
       </c>
     </row>
     <row r="24">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2570.37</v>
+        <v>2311.13</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
@@ -976,7 +976,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>prom 856.79</t>
+          <t>prom 770.38</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>48852.99</v>
+        <v>42423.82</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -997,7 +997,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>prom 16284.33</t>
+          <t>prom 14141.27</t>
         </is>
       </c>
     </row>
@@ -1008,17 +1008,17 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1033.16</v>
+        <v>935.0599999999999</v>
       </c>
       <c r="C28" t="n">
-        <v>51079.14</v>
+        <v>788888.89</v>
       </c>
       <c r="D28" t="n">
-        <v>237704.92</v>
+        <v>190789.47</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>prom 96605.74</t>
+          <t>prom 326871.14</t>
         </is>
       </c>
     </row>
@@ -1029,17 +1029,17 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>140316.69</v>
+        <v>130909.09</v>
       </c>
       <c r="C29" t="n">
-        <v>53787.88</v>
+        <v>887500</v>
       </c>
       <c r="D29" t="n">
-        <v>329545.45</v>
+        <v>302083.33</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>prom 174550.01</t>
+          <t>prom 440164.14</t>
         </is>
       </c>
     </row>
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>171785360</v>
+        <v>201110465</v>
       </c>
       <c r="C30" t="n">
-        <v>5706000</v>
+        <v>146800</v>
       </c>
       <c r="D30" t="n">
-        <v>1993150</v>
+        <v>2030750</v>
       </c>
       <c r="E30" t="n">
-        <v>179484510</v>
+        <v>203288015</v>
       </c>
     </row>
     <row r="31">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>262.51</v>
+        <v>324.4</v>
       </c>
     </row>
     <row r="32">
@@ -1079,16 +1079,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>140717445</v>
+        <v>151078375</v>
       </c>
       <c r="C32" t="n">
-        <v>20668800</v>
+        <v>431000</v>
       </c>
       <c r="D32" t="n">
-        <v>9992590</v>
+        <v>10706650</v>
       </c>
       <c r="E32" t="n">
-        <v>171378835</v>
+        <v>162216025</v>
       </c>
     </row>
     <row r="33">
@@ -1098,13 +1098,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>22.15</v>
+        <v>31.14</v>
       </c>
       <c r="C33" t="n">
-        <v>191.11</v>
+        <v>-93.93000000000001</v>
       </c>
       <c r="D33" t="n">
-        <v>-31.09</v>
+        <v>-26.16</v>
       </c>
     </row>
   </sheetData>
@@ -1168,13 +1168,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5708</v>
+        <v>6863</v>
       </c>
       <c r="D2" t="n">
-        <v>361</v>
+        <v>432</v>
       </c>
       <c r="E2" t="n">
-        <v>6.32</v>
+        <v>6.29</v>
       </c>
     </row>
     <row r="3">
@@ -1189,13 +1189,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>197780</v>
+        <v>210543</v>
       </c>
       <c r="D3" t="n">
-        <v>958</v>
+        <v>989</v>
       </c>
       <c r="E3" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="4">
@@ -1210,13 +1210,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>39920</v>
+        <v>41669</v>
       </c>
       <c r="D4" t="n">
-        <v>1203</v>
+        <v>1325</v>
       </c>
       <c r="E4" t="n">
-        <v>3.01</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="5">
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43252</v>
+        <v>46174</v>
       </c>
       <c r="D5" t="n">
-        <v>4498</v>
+        <v>5234</v>
       </c>
       <c r="E5" t="n">
-        <v>10.4</v>
+        <v>11.34</v>
       </c>
     </row>
     <row r="6">
@@ -1252,13 +1252,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>98.18000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>145</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>135</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>93.09999999999999</v>
+        <v>81.81999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1294,13 +1294,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>84.62</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="9">
@@ -1315,13 +1315,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>377</v>
+        <v>10</v>
       </c>
       <c r="D9" t="n">
-        <v>370</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>98.14</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10">
@@ -1336,13 +1336,13 @@
         </is>
       </c>
       <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
         <v>4</v>
       </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
       <c r="E10" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="D11" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E11" t="n">
-        <v>69.7</v>
+        <v>61.73</v>
       </c>
     </row>
     <row r="12">
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>52.94</v>
+        <v>52.63</v>
       </c>
     </row>
     <row r="13">
@@ -1402,10 +1402,10 @@
         <v>40</v>
       </c>
       <c r="D13" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E13" t="n">
-        <v>87.5</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1475,10 +1475,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>369148</v>
+        <v>398556</v>
       </c>
       <c r="D2" t="n">
-        <v>369148</v>
+        <v>398556</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1501,10 +1501,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>286660</v>
+        <v>305249</v>
       </c>
       <c r="D3" t="n">
-        <v>286660</v>
+        <v>305249</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1528,11 +1528,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>&lt;= 286660</t>
+          <t>&lt;= 305249</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>152231</v>
+        <v>170085</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1556,11 +1556,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>&lt;= 152231</t>
+          <t>&lt;= 170085</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5892</v>
+        <v>6911</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.87%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1611,11 +1611,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>&gt;= 5892</t>
+          <t>&gt;= 6911</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8755</v>
+        <v>9525</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -1638,10 +1638,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>965</v>
+        <v>44</v>
       </c>
       <c r="D8" t="n">
-        <v>965</v>
+        <v>44</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -1664,10 +1664,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>616</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>616</v>
+        <v>25</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1691,11 +1691,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>&lt;= 616</t>
+          <t>&lt;= 25</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>600</v>
+        <v>21</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1719,11 +1719,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>&lt;= 600</t>
+          <t>&lt;= 21</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>581</v>
+        <v>18</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>96.83%</t>
+          <t>85.71%</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1774,11 +1774,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>&gt;= 581</t>
+          <t>&gt;= 18</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>864</v>
+        <v>94</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="D14" t="n">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -1827,10 +1827,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="D15" t="n">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -1854,11 +1854,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;= 127</t>
+          <t>&lt;= 145</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,11 +1882,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>&lt;= 105</t>
+          <t>&lt;= 123</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>73.33%</t>
+          <t>68.29%</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>&gt;= 77</t>
+          <t>&gt;= 84</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>96.83%</t>
+          <t>85.71%</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>73.33%</t>
+          <t>68.29%</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -2263,34 +2263,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>369148</v>
+        <v>398556</v>
       </c>
       <c r="C2" t="n">
-        <v>11468</v>
+        <v>13170</v>
       </c>
       <c r="D2" t="n">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="E2" t="n">
-        <v>357492</v>
+        <v>385231</v>
       </c>
       <c r="F2" t="n">
-        <v>369148</v>
+        <v>398556</v>
       </c>
       <c r="G2" t="n">
-        <v>286660</v>
+        <v>305249</v>
       </c>
       <c r="H2" t="n">
-        <v>7020</v>
+        <v>7980</v>
       </c>
       <c r="I2" t="n">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="J2" t="n">
-        <v>279452</v>
+        <v>297114</v>
       </c>
       <c r="K2" t="n">
-        <v>286660</v>
+        <v>305249</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -2303,34 +2303,34 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>152231</v>
+        <v>170085</v>
       </c>
       <c r="O2" t="n">
-        <v>5892</v>
+        <v>6911</v>
       </c>
       <c r="P2" t="n">
-        <v>3.8704</v>
+        <v>4.0633</v>
       </c>
       <c r="Q2" t="n">
-        <v>8755</v>
+        <v>9525</v>
       </c>
       <c r="R2" t="n">
-        <v>6926</v>
+        <v>7993</v>
       </c>
       <c r="S2" t="n">
-        <v>1641</v>
+        <v>1377</v>
       </c>
       <c r="T2" t="n">
-        <v>18436</v>
+        <v>20504</v>
       </c>
       <c r="U2" t="n">
-        <v>970</v>
+        <v>1117</v>
       </c>
       <c r="V2" t="n">
-        <v>111503</v>
+        <v>123201</v>
       </c>
       <c r="W2" t="n">
-        <v>821</v>
+        <v>880</v>
       </c>
       <c r="X2" t="n">
         <v>47387402.9</v>
@@ -2339,28 +2339,28 @@
         <v>115200000</v>
       </c>
       <c r="Z2" t="n">
-        <v>2570.37</v>
+        <v>2311.13</v>
       </c>
       <c r="AA2" t="n">
-        <v>48852.99</v>
+        <v>42423.82</v>
       </c>
       <c r="AB2" t="n">
-        <v>1033.16</v>
+        <v>935.0599999999999</v>
       </c>
       <c r="AC2" t="n">
-        <v>140316.69</v>
+        <v>130909.09</v>
       </c>
       <c r="AD2" t="n">
-        <v>171785360</v>
+        <v>201110465</v>
       </c>
       <c r="AE2" t="n">
-        <v>262.51</v>
+        <v>324.4</v>
       </c>
       <c r="AF2" t="n">
-        <v>140717445</v>
+        <v>151078375</v>
       </c>
       <c r="AG2" t="n">
-        <v>22.15</v>
+        <v>31.14</v>
       </c>
     </row>
     <row r="3">
@@ -2370,34 +2370,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>965</v>
+        <v>44</v>
       </c>
       <c r="C3" t="n">
-        <v>941</v>
+        <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>965</v>
+        <v>44</v>
       </c>
       <c r="G3" t="n">
-        <v>616</v>
+        <v>25</v>
       </c>
       <c r="H3" t="n">
-        <v>592</v>
+        <v>21</v>
       </c>
       <c r="I3" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>616</v>
+        <v>25</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -2410,34 +2410,34 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>600</v>
+        <v>21</v>
       </c>
       <c r="O3" t="n">
-        <v>581</v>
+        <v>18</v>
       </c>
       <c r="P3" t="n">
-        <v>96.83329999999999</v>
+        <v>85.71429999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>864</v>
+        <v>94</v>
       </c>
       <c r="R3" t="n">
-        <v>572</v>
+        <v>19</v>
       </c>
       <c r="S3" t="n">
-        <v>268</v>
+        <v>71</v>
       </c>
       <c r="T3" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="U3" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="V3" t="n">
-        <v>139</v>
+        <v>9</v>
       </c>
       <c r="W3" t="n">
-        <v>132</v>
+        <v>8</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
@@ -2452,19 +2452,19 @@
         <v>0</v>
       </c>
       <c r="AB3" t="n">
-        <v>51079.14</v>
+        <v>788888.89</v>
       </c>
       <c r="AC3" t="n">
-        <v>53787.88</v>
+        <v>887500</v>
       </c>
       <c r="AD3" t="n">
-        <v>5706000</v>
+        <v>146800</v>
       </c>
       <c r="AF3" t="n">
-        <v>20668800</v>
+        <v>431000</v>
       </c>
       <c r="AG3" t="n">
-        <v>191.11</v>
+        <v>-93.93000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -2474,74 +2474,74 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="C4" t="n">
+        <v>133</v>
+      </c>
+      <c r="D4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>178</v>
+      </c>
+      <c r="G4" t="n">
+        <v>145</v>
+      </c>
+      <c r="H4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="n">
+        <v>45</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>145</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
         <v>123</v>
       </c>
-      <c r="D4" t="n">
-        <v>34</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>157</v>
-      </c>
-      <c r="G4" t="n">
-        <v>127</v>
-      </c>
-      <c r="H4" t="n">
-        <v>93</v>
-      </c>
-      <c r="I4" t="n">
-        <v>34</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>127</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-02-14</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>105</v>
-      </c>
       <c r="O4" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="P4" t="n">
-        <v>73.33329999999999</v>
+        <v>68.2927</v>
       </c>
       <c r="Q4" t="n">
         <v>325</v>
       </c>
       <c r="R4" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="S4" t="n">
-        <v>239</v>
+        <v>222</v>
       </c>
       <c r="T4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="U4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V4" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="W4" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
@@ -2556,19 +2556,19 @@
         <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>237704.92</v>
+        <v>190789.47</v>
       </c>
       <c r="AC4" t="n">
-        <v>329545.45</v>
+        <v>302083.33</v>
       </c>
       <c r="AD4" t="n">
-        <v>1993150</v>
+        <v>2030750</v>
       </c>
       <c r="AF4" t="n">
-        <v>9992590</v>
+        <v>10706650</v>
       </c>
       <c r="AG4" t="n">
-        <v>-31.09</v>
+        <v>-26.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>